<commit_message>
atualizei os dados do 2Q26 da OKLO
</commit_message>
<xml_diff>
--- a/analise_eua/energia_eletrica/oklo/oklo_indicators.xlsx
+++ b/analise_eua/energia_eletrica/oklo/oklo_indicators.xlsx
@@ -755,7 +755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AB3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -897,88 +897,174 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46112</v>
+        <v>46203</v>
       </c>
       <c r="B2" t="n">
-        <v>-255.46</v>
+        <v>-190</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-72853</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-4011.24</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="H2" t="n">
+        <v>9221823383.996523</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3259</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2465158</v>
+      </c>
+      <c r="K2" t="n">
+        <v>-2461899</v>
+      </c>
+      <c r="L2" t="n">
+        <v>13.09</v>
+      </c>
+      <c r="M2" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-62.14</v>
+      </c>
+      <c r="O2" t="n">
+        <v>-4.15</v>
+      </c>
+      <c r="P2" t="n">
+        <v>-5.73</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>-47592</v>
+      </c>
+      <c r="R2" t="n">
+        <v>-553697</v>
+      </c>
+      <c r="S2" t="n">
+        <v>668790</v>
+      </c>
+      <c r="T2" t="n">
+        <v>-115947</v>
+      </c>
+      <c r="U2" t="n">
+        <v>68355</v>
+      </c>
+      <c r="V2" t="n">
+        <v>106339</v>
+      </c>
+      <c r="W2" t="n">
+        <v>39474</v>
+      </c>
+      <c r="X2" t="n">
+        <v>199275</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>2468892</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>-114.23</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>-257604</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>-321873</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-255.46</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
         <v>-0.89</v>
       </c>
-      <c r="E2" t="n">
-        <v>163</v>
-      </c>
-      <c r="F2" t="n">
+      <c r="E3" t="n">
+        <v>-51086</v>
+      </c>
+      <c r="F3" t="n">
         <v>0</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G3" t="n">
         <v>3.2</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H3" t="n">
         <v>8446850490.130868</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I3" t="n">
         <v>2620</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J3" t="n">
         <v>2208609</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K3" t="n">
         <v>-2205989</v>
       </c>
-      <c r="L2" t="n">
-        <v>-4115.65</v>
-      </c>
-      <c r="M2" t="n">
+      <c r="L3" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="M3" t="n">
         <v>-0.84</v>
       </c>
-      <c r="N2" t="n">
-        <v>19874.7</v>
-      </c>
-      <c r="O2" t="n">
+      <c r="N3" t="n">
+        <v>-80.15000000000001</v>
+      </c>
+      <c r="O3" t="n">
         <v>-3.69</v>
       </c>
-      <c r="P2" t="n">
-        <v>-0.01</v>
-      </c>
-      <c r="Q2" t="n">
+      <c r="P3" t="n">
+        <v>-5.06</v>
+      </c>
+      <c r="Q3" t="n">
         <v>-17867</v>
       </c>
-      <c r="R2" t="n">
+      <c r="R3" t="n">
         <v>-359034</v>
       </c>
-      <c r="S2" t="n">
+      <c r="S3" t="n">
         <v>1182559</v>
       </c>
-      <c r="T2" t="n">
+      <c r="T3" t="n">
         <v>-50677</v>
       </c>
-      <c r="U2" t="n">
+      <c r="U3" t="n">
         <v>32810</v>
       </c>
-      <c r="V2" t="n">
+      <c r="V3" t="n">
         <v>39429</v>
       </c>
-      <c r="W2" t="n">
+      <c r="W3" t="n">
         <v>27049</v>
       </c>
-      <c r="X2" t="n">
+      <c r="X3" t="n">
         <v>100737</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Y3" t="n">
         <v>2188522</v>
       </c>
-      <c r="Z2" t="n">
-        <v>-34404.76</v>
-      </c>
-      <c r="AA2" t="n">
+      <c r="Z3" t="n">
+        <v>-75.63</v>
+      </c>
+      <c r="AA3" t="n">
         <v>-137124</v>
       </c>
-      <c r="AB2" t="n">
-        <v>-39842</v>
+      <c r="AB3" t="n">
+        <v>-173289</v>
       </c>
     </row>
   </sheetData>

</xml_diff>